<commit_message>
feat: export fee workbooks as xlsx templates
</commit_message>
<xml_diff>
--- a/outputs/ema-fee-export-template/EMA费用导出模板.xlsx
+++ b/outputs/ema-fee-export-template/EMA费用导出模板.xlsx
@@ -57,13 +57,30 @@
     <definedName name="_PT_FORECAST_PROTO_ADDITIONAL" hidden="1">'费用预估'!$A$135:$W$135</definedName>
     <definedName name="_PT_SGS_DYNAMIC_START" hidden="1">'SGS'!$A$6</definedName>
     <definedName name="_PT_SGS_DYNAMIC_END" hidden="1">'SGS'!$R$175</definedName>
+    <definedName name="_PT_SGS_PROTO_PHASE" hidden="1">'SGS'!$A$6:$R$6</definedName>
+    <definedName name="_PT_SGS_PROTO_GROUP" hidden="1">'SGS'!$A$7:$R$7</definedName>
+    <definedName name="_PT_SGS_PROTO_HEADER" hidden="1">'SGS'!$A$8:$R$8</definedName>
     <definedName name="_PT_SGS_PROTO_DATA" hidden="1">'SGS'!$A$9:$R$9</definedName>
+    <definedName name="_PT_SGS_PROTO_TOTAL" hidden="1">'SGS'!$A$27:$R$27</definedName>
     <definedName name="_PT_CTI_DYNAMIC_START" hidden="1">'华测'!$A$6</definedName>
     <definedName name="_PT_CTI_DYNAMIC_END" hidden="1">'华测'!$R$174</definedName>
+    <definedName name="_PT_CTI_PROTO_PHASE" hidden="1">'华测'!$A$6:$R$6</definedName>
+    <definedName name="_PT_CTI_PROTO_GROUP" hidden="1">'华测'!$A$7:$R$7</definedName>
+    <definedName name="_PT_CTI_PROTO_HEADER" hidden="1">'华测'!$A$8:$R$8</definedName>
     <definedName name="_PT_CTI_PROTO_DATA" hidden="1">'华测'!$A$9:$R$9</definedName>
+    <definedName name="_PT_CTI_PROTO_TOTAL" hidden="1">'华测'!$A$27:$R$27</definedName>
     <definedName name="_PT_SUBO_DYNAMIC_START" hidden="1">'苏勃'!$A$6</definedName>
     <definedName name="_PT_SUBO_DYNAMIC_END" hidden="1">'苏勃'!$R$174</definedName>
+    <definedName name="_PT_SUBO_PROTO_PHASE" hidden="1">'苏勃'!$A$6:$R$6</definedName>
+    <definedName name="_PT_SUBO_PROTO_GROUP" hidden="1">'苏勃'!$A$7:$R$7</definedName>
+    <definedName name="_PT_SUBO_PROTO_HEADER" hidden="1">'苏勃'!$A$8:$R$8</definedName>
     <definedName name="_PT_SUBO_PROTO_DATA" hidden="1">'苏勃'!$A$9:$R$9</definedName>
+    <definedName name="_PT_SUBO_PROTO_TOTAL" hidden="1">'苏勃'!$A$27:$R$27</definedName>
+    <definedName name="_PT_COMPARE_DYNAMIC_START" hidden="1">'费用对比'!$A$9</definedName>
+    <definedName name="_PT_COMPARE_DYNAMIC_END" hidden="1">'费用对比'!$R$37</definedName>
+    <definedName name="_PT_COMPARE_PROTO_PHASE" hidden="1">'费用对比'!$A$9:$R$9</definedName>
+    <definedName name="_PT_COMPARE_PROTO_HEADER" hidden="1">'费用对比'!$A$11:$R$11</definedName>
+    <definedName name="_PT_COMPARE_PROTO_DATA" hidden="1">'费用对比'!$A$12:$R$12</definedName>
     <definedName name="_PT_COMPARE_HELPER_RANGE" hidden="1">'费用对比'!$S$1:$X$15</definedName>
     <definedName name="_PT_SPECIAL_DYNAMIC_START" hidden="1">'特殊项目费用'!$A$9</definedName>
     <definedName name="_PT_SPECIAL_DYNAMIC_END" hidden="1">'特殊项目费用'!$M$37</definedName>

</xml_diff>